<commit_message>
Added source files and py script to convert to yaml. Modiefied yaml with methods.
</commit_message>
<xml_diff>
--- a/source_files/_analytical methods.xlsx
+++ b/source_files/_analytical methods.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucnmuni-my.sharepoint.com/personal/63543_muni_cz/Documents/CRA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\269713\GitHub\cra_analytical_methods_vocabulary\source_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F3723D8-AF11-43A3-9651-1B1CB9FAA023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABD0A5B5-BFDA-4DA4-9190-D20512C9610D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="45600" windowHeight="18960" xr2:uid="{BC79B45B-7914-4D87-9A96-0220A5CD89B6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{BC79B45B-7914-4D87-9A96-0220A5CD89B6}"/>
   </bookViews>
   <sheets>
     <sheet name="analytical method" sheetId="3" r:id="rId1"/>
     <sheet name="analytical method groupping" sheetId="7" r:id="rId2"/>
+    <sheet name="methods-vocabulary" sheetId="8" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'analytical method'!$A$1:$D$103</definedName>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="908" uniqueCount="262">
   <si>
     <t>analytical method group</t>
   </si>
@@ -490,13 +491,349 @@
   </si>
   <si>
     <t>LC-NMR</t>
+  </si>
+  <si>
+    <t>F_AAS</t>
+  </si>
+  <si>
+    <t>GF_AAS</t>
+  </si>
+  <si>
+    <t>CV_AAS</t>
+  </si>
+  <si>
+    <t>TDA_AAS</t>
+  </si>
+  <si>
+    <t>F_AES</t>
+  </si>
+  <si>
+    <t>GD_AES</t>
+  </si>
+  <si>
+    <t>HG_AFS</t>
+  </si>
+  <si>
+    <t>FI_AFS</t>
+  </si>
+  <si>
+    <t>CV_AFS</t>
+  </si>
+  <si>
+    <t>ICP_AES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICP_OES </t>
+  </si>
+  <si>
+    <t>1H_NMR</t>
+  </si>
+  <si>
+    <t>13C_NMR</t>
+  </si>
+  <si>
+    <t>UV_Vis</t>
+  </si>
+  <si>
+    <t>ICP_MS</t>
+  </si>
+  <si>
+    <t>ICP_DRC_MS</t>
+  </si>
+  <si>
+    <t>ICP_KED_MS</t>
+  </si>
+  <si>
+    <t>GC_MS</t>
+  </si>
+  <si>
+    <t>GC_HRMS</t>
+  </si>
+  <si>
+    <t>GC_EI_MS</t>
+  </si>
+  <si>
+    <t>GC_EI_HRMS</t>
+  </si>
+  <si>
+    <t>GC_NCI_MS</t>
+  </si>
+  <si>
+    <t>GC_NCI_HRMS</t>
+  </si>
+  <si>
+    <t>GC_CI_MS</t>
+  </si>
+  <si>
+    <t>GC_CI_HRMS</t>
+  </si>
+  <si>
+    <t>GC_APPI_MS</t>
+  </si>
+  <si>
+    <t>GC_APPI_HRMS</t>
+  </si>
+  <si>
+    <t>GC_APCI_MS</t>
+  </si>
+  <si>
+    <t>GC_APCI_HRMS</t>
+  </si>
+  <si>
+    <t>GC×GC_MS</t>
+  </si>
+  <si>
+    <t>GC×GC_HRMS</t>
+  </si>
+  <si>
+    <t>LC_MS</t>
+  </si>
+  <si>
+    <t>LC_HRMS</t>
+  </si>
+  <si>
+    <t>HPLC_MS</t>
+  </si>
+  <si>
+    <t>HPLC_HRMS</t>
+  </si>
+  <si>
+    <t>UPLC_MS</t>
+  </si>
+  <si>
+    <t>UPLC_HRMS</t>
+  </si>
+  <si>
+    <t>IC_MS</t>
+  </si>
+  <si>
+    <t>IC_HRMS</t>
+  </si>
+  <si>
+    <t>IC_ESI_MS</t>
+  </si>
+  <si>
+    <t>IC_ESI_HRMS</t>
+  </si>
+  <si>
+    <t>SFC_MS</t>
+  </si>
+  <si>
+    <t>SFC_HRMS</t>
+  </si>
+  <si>
+    <t>LC_DAD</t>
+  </si>
+  <si>
+    <t>LC_FLD</t>
+  </si>
+  <si>
+    <t>LC_UV</t>
+  </si>
+  <si>
+    <t>HPLC_DAD</t>
+  </si>
+  <si>
+    <t>HPLC_FLD</t>
+  </si>
+  <si>
+    <t>HPLC_UV</t>
+  </si>
+  <si>
+    <t>UPLC_DAD</t>
+  </si>
+  <si>
+    <t>UPLC_FLD</t>
+  </si>
+  <si>
+    <t>UPLC_UV</t>
+  </si>
+  <si>
+    <t>GC_ECD</t>
+  </si>
+  <si>
+    <t>GC_FID</t>
+  </si>
+  <si>
+    <t>GC_PID</t>
+  </si>
+  <si>
+    <t>IC_UV</t>
+  </si>
+  <si>
+    <t>IC_DAD</t>
+  </si>
+  <si>
+    <t>IC_FLD</t>
+  </si>
+  <si>
+    <t>LC_ICP_MS</t>
+  </si>
+  <si>
+    <t>GC_ICP_MS</t>
+  </si>
+  <si>
+    <t>IC_ICP_MS</t>
+  </si>
+  <si>
+    <t>LC_IR</t>
+  </si>
+  <si>
+    <t>LC_NMR</t>
+  </si>
+  <si>
+    <t>UV_Vis _ DAD</t>
+  </si>
+  <si>
+    <t>ICP_MS_MS</t>
+  </si>
+  <si>
+    <t>GC_MS_MS</t>
+  </si>
+  <si>
+    <t>GC_HRMS_MS</t>
+  </si>
+  <si>
+    <t>GC_EI_MS_MS</t>
+  </si>
+  <si>
+    <t>GC_EI_HRMS_MS</t>
+  </si>
+  <si>
+    <t>GC_NCI_MS_MS</t>
+  </si>
+  <si>
+    <t>GC_NCI_HRMS_MS</t>
+  </si>
+  <si>
+    <t>GC_CI_MS_MS</t>
+  </si>
+  <si>
+    <t>GC_CI_HRMS_MS</t>
+  </si>
+  <si>
+    <t>GC_APPI_MS_MS</t>
+  </si>
+  <si>
+    <t>GC_APPI_HRMS_MS</t>
+  </si>
+  <si>
+    <t>GC_APCI_MS_MS</t>
+  </si>
+  <si>
+    <t>GC_APCI_HRMS_MS</t>
+  </si>
+  <si>
+    <t>GC×GC_MS_MS</t>
+  </si>
+  <si>
+    <t>LC_MS_MS</t>
+  </si>
+  <si>
+    <t>LC_HRMS_MS</t>
+  </si>
+  <si>
+    <t>HPLC_MS_MS</t>
+  </si>
+  <si>
+    <t>HPLC_HRMS_MS</t>
+  </si>
+  <si>
+    <t>UPLC_MS_MS</t>
+  </si>
+  <si>
+    <t>UPLC_HRMS_MS</t>
+  </si>
+  <si>
+    <t>IC_MS_MS</t>
+  </si>
+  <si>
+    <t>IC_HRMS_MS</t>
+  </si>
+  <si>
+    <t>IC_ESI_MS_MS</t>
+  </si>
+  <si>
+    <t>IC_ESI_HRMS_MS</t>
+  </si>
+  <si>
+    <t>SFC_MS_MS</t>
+  </si>
+  <si>
+    <t>SFC_HRMS_MS</t>
+  </si>
+  <si>
+    <t>LC_ICP_MS_MS</t>
+  </si>
+  <si>
+    <t>aas</t>
+  </si>
+  <si>
+    <t>aes</t>
+  </si>
+  <si>
+    <t>afs</t>
+  </si>
+  <si>
+    <t>icp</t>
+  </si>
+  <si>
+    <t>icpms</t>
+  </si>
+  <si>
+    <t>xrf</t>
+  </si>
+  <si>
+    <t>nmr</t>
+  </si>
+  <si>
+    <t>uvvis</t>
+  </si>
+  <si>
+    <t>gcms</t>
+  </si>
+  <si>
+    <t>lcms</t>
+  </si>
+  <si>
+    <t>icms</t>
+  </si>
+  <si>
+    <t>sfc</t>
+  </si>
+  <si>
+    <t>lc</t>
+  </si>
+  <si>
+    <t>gc</t>
+  </si>
+  <si>
+    <t>ic</t>
+  </si>
+  <si>
+    <t>mixedicp</t>
+  </si>
+  <si>
+    <t>mixothers</t>
+  </si>
+  <si>
+    <t>parent_method</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>name alter</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -879,17 +1216,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D289B77-1EF5-4CBC-8132-594E1A5C4EEF}">
   <dimension ref="A1:D103"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.140625" customWidth="1"/>
-    <col min="2" max="2" width="57.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.140625" customWidth="1"/>
-    <col min="4" max="4" width="29.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.1796875" customWidth="1"/>
+    <col min="2" max="2" width="57.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.1796875" customWidth="1"/>
+    <col min="4" max="4" width="29.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.81640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="83" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -903,7 +1240,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -914,7 +1251,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -928,7 +1265,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -942,7 +1279,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -956,7 +1293,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -970,7 +1307,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -984,7 +1321,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -998,7 +1335,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1012,7 +1349,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1026,7 +1363,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1040,7 +1377,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1054,7 +1391,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -1068,7 +1405,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1082,7 +1419,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -1096,7 +1433,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -1110,7 +1447,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -1124,7 +1461,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>4</v>
       </c>
@@ -1138,7 +1475,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>4</v>
       </c>
@@ -1152,7 +1489,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>4</v>
       </c>
@@ -1166,7 +1503,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>4</v>
       </c>
@@ -1180,7 +1517,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>4</v>
       </c>
@@ -1194,7 +1531,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>4</v>
       </c>
@@ -1208,7 +1545,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>4</v>
       </c>
@@ -1222,7 +1559,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>4</v>
       </c>
@@ -1236,7 +1573,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>59</v>
       </c>
@@ -1247,7 +1584,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>59</v>
       </c>
@@ -1258,7 +1595,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -1269,7 +1606,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -1280,7 +1617,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>59</v>
       </c>
@@ -1291,7 +1628,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>59</v>
       </c>
@@ -1302,7 +1639,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>59</v>
       </c>
@@ -1313,7 +1650,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>59</v>
       </c>
@@ -1324,7 +1661,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>59</v>
       </c>
@@ -1335,7 +1672,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>59</v>
       </c>
@@ -1346,7 +1683,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>59</v>
       </c>
@@ -1357,7 +1694,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>59</v>
       </c>
@@ -1368,7 +1705,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>59</v>
       </c>
@@ -1379,7 +1716,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>59</v>
       </c>
@@ -1390,7 +1727,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>59</v>
       </c>
@@ -1401,7 +1738,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>59</v>
       </c>
@@ -1412,7 +1749,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>59</v>
       </c>
@@ -1423,7 +1760,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>59</v>
       </c>
@@ -1434,7 +1771,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>59</v>
       </c>
@@ -1445,7 +1782,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>59</v>
       </c>
@@ -1456,7 +1793,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>59</v>
       </c>
@@ -1467,7 +1804,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>59</v>
       </c>
@@ -1478,7 +1815,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>59</v>
       </c>
@@ -1489,7 +1826,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>59</v>
       </c>
@@ -1500,7 +1837,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>59</v>
       </c>
@@ -1511,7 +1848,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>59</v>
       </c>
@@ -1522,7 +1859,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="52" spans="1:3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>59</v>
       </c>
@@ -1533,7 +1870,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>59</v>
       </c>
@@ -1544,7 +1881,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>59</v>
       </c>
@@ -1555,7 +1892,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="55" spans="1:3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>59</v>
       </c>
@@ -1566,7 +1903,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="56" spans="1:3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>59</v>
       </c>
@@ -1577,7 +1914,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="57" spans="1:3">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>59</v>
       </c>
@@ -1588,7 +1925,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="58" spans="1:3">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>59</v>
       </c>
@@ -1599,7 +1936,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="59" spans="1:3">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>59</v>
       </c>
@@ -1610,7 +1947,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="60" spans="1:3">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>59</v>
       </c>
@@ -1621,7 +1958,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="61" spans="1:3">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>59</v>
       </c>
@@ -1632,7 +1969,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="62" spans="1:3">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>59</v>
       </c>
@@ -1643,7 +1980,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="63" spans="1:3">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>59</v>
       </c>
@@ -1654,7 +1991,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="64" spans="1:3">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>59</v>
       </c>
@@ -1665,7 +2002,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="65" spans="1:3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>59</v>
       </c>
@@ -1676,7 +2013,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="66" spans="1:3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>59</v>
       </c>
@@ -1687,7 +2024,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="67" spans="1:3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>59</v>
       </c>
@@ -1698,7 +2035,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="68" spans="1:3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>59</v>
       </c>
@@ -1709,7 +2046,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="69" spans="1:3">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>59</v>
       </c>
@@ -1720,7 +2057,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="70" spans="1:3">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>59</v>
       </c>
@@ -1731,7 +2068,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="71" spans="1:3">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>59</v>
       </c>
@@ -1742,7 +2079,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="72" spans="1:3">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>59</v>
       </c>
@@ -1753,7 +2090,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="73" spans="1:3">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>59</v>
       </c>
@@ -1764,7 +2101,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="74" spans="1:3">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>59</v>
       </c>
@@ -1775,7 +2112,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="75" spans="1:3">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>59</v>
       </c>
@@ -1786,7 +2123,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="76" spans="1:3">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>59</v>
       </c>
@@ -1797,7 +2134,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="77" spans="1:3">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>59</v>
       </c>
@@ -1808,7 +2145,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="78" spans="1:3">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>59</v>
       </c>
@@ -1819,7 +2156,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="79" spans="1:3">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>59</v>
       </c>
@@ -1830,7 +2167,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="80" spans="1:3">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>59</v>
       </c>
@@ -1841,7 +2178,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="81" spans="1:3">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>120</v>
       </c>
@@ -1852,7 +2189,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="82" spans="1:3">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>120</v>
       </c>
@@ -1863,7 +2200,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="83" spans="1:3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>120</v>
       </c>
@@ -1874,7 +2211,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="84" spans="1:3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>120</v>
       </c>
@@ -1885,7 +2222,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="85" spans="1:3">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>120</v>
       </c>
@@ -1896,7 +2233,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="86" spans="1:3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>120</v>
       </c>
@@ -1907,7 +2244,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="87" spans="1:3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>120</v>
       </c>
@@ -1918,7 +2255,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="88" spans="1:3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>120</v>
       </c>
@@ -1929,7 +2266,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="89" spans="1:3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>120</v>
       </c>
@@ -1940,7 +2277,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="90" spans="1:3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>120</v>
       </c>
@@ -1951,7 +2288,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="91" spans="1:3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>120</v>
       </c>
@@ -1962,7 +2299,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="92" spans="1:3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>120</v>
       </c>
@@ -1973,7 +2310,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="93" spans="1:3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>120</v>
       </c>
@@ -1984,7 +2321,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="94" spans="1:3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>120</v>
       </c>
@@ -1995,7 +2332,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="95" spans="1:3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>120</v>
       </c>
@@ -2006,7 +2343,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="96" spans="1:3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>120</v>
       </c>
@@ -2017,7 +2354,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="97" spans="1:3">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>120</v>
       </c>
@@ -2028,7 +2365,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="98" spans="1:3">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>141</v>
       </c>
@@ -2039,7 +2376,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="99" spans="1:3">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>141</v>
       </c>
@@ -2050,7 +2387,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="100" spans="1:3">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>141</v>
       </c>
@@ -2061,7 +2398,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="101" spans="1:3">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>141</v>
       </c>
@@ -2072,7 +2409,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="102" spans="1:3">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>141</v>
       </c>
@@ -2083,7 +2420,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="103" spans="1:3">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>141</v>
       </c>
@@ -2104,13 +2441,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{087FBFDD-59F6-406E-8F7C-E67A59E5FA1F}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.7109375" customWidth="1"/>
-    <col min="2" max="2" width="57.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.7265625" customWidth="1"/>
+    <col min="2" max="2" width="57.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2118,7 +2455,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2126,7 +2463,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -2134,7 +2471,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -2142,7 +2479,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -2150,7 +2487,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -2158,7 +2495,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -2166,7 +2503,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -2174,7 +2511,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>59</v>
       </c>
@@ -2182,7 +2519,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -2190,7 +2527,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>59</v>
       </c>
@@ -2198,7 +2535,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>59</v>
       </c>
@@ -2206,7 +2543,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>59</v>
       </c>
@@ -2214,7 +2551,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>120</v>
       </c>
@@ -2222,7 +2559,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>120</v>
       </c>
@@ -2230,7 +2567,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>120</v>
       </c>
@@ -2238,7 +2575,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>141</v>
       </c>
@@ -2246,12 +2583,1853 @@
         <v>142</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>141</v>
       </c>
       <c r="B18" t="s">
         <v>147</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D056ED3-D42E-40D3-8F50-ADCBF2D92FDA}">
+  <dimension ref="A1:F103"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="21.90625" customWidth="1"/>
+    <col min="2" max="2" width="46.26953125" customWidth="1"/>
+    <col min="3" max="3" width="32" customWidth="1"/>
+    <col min="4" max="4" width="26.08984375" customWidth="1"/>
+    <col min="5" max="5" width="32.90625" customWidth="1"/>
+    <col min="6" max="6" width="26.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>258</v>
+      </c>
+      <c r="D1" t="s">
+        <v>261</v>
+      </c>
+      <c r="E1" t="s">
+        <v>260</v>
+      </c>
+      <c r="F1" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>241</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>241</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>241</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>241</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>241</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>241</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
+        <v>242</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" t="s">
+        <v>242</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" t="s">
+        <v>242</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>242</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>243</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>243</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" t="s">
+        <v>32</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>243</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>243</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" t="s">
+        <v>36</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" t="s">
+        <v>244</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E17" t="s">
+        <v>39</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" t="s">
+        <v>244</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E18" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" t="s">
+        <v>246</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E19" t="s">
+        <v>44</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" t="s">
+        <v>246</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E20" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" t="s">
+        <v>246</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E21" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
+        <v>49</v>
+      </c>
+      <c r="C22" t="s">
+        <v>247</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E22" t="s">
+        <v>51</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" t="s">
+        <v>247</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E23" t="s">
+        <v>53</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" t="s">
+        <v>248</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E24" t="s">
+        <v>56</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" t="s">
+        <v>248</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E25" t="s">
+        <v>58</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>59</v>
+      </c>
+      <c r="B26" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" t="s">
+        <v>245</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B27" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" t="s">
+        <v>245</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>59</v>
+      </c>
+      <c r="B28" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28" t="s">
+        <v>245</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>59</v>
+      </c>
+      <c r="B29" t="s">
+        <v>60</v>
+      </c>
+      <c r="C29" t="s">
+        <v>245</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>59</v>
+      </c>
+      <c r="B30" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" t="s">
+        <v>249</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>59</v>
+      </c>
+      <c r="B31" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" t="s">
+        <v>249</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>59</v>
+      </c>
+      <c r="B32" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" t="s">
+        <v>249</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>59</v>
+      </c>
+      <c r="B33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C33" t="s">
+        <v>249</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" t="s">
+        <v>249</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>59</v>
+      </c>
+      <c r="B35" t="s">
+        <v>65</v>
+      </c>
+      <c r="C35" t="s">
+        <v>249</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>59</v>
+      </c>
+      <c r="B36" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" t="s">
+        <v>249</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>59</v>
+      </c>
+      <c r="B37" t="s">
+        <v>65</v>
+      </c>
+      <c r="C37" t="s">
+        <v>249</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38" t="s">
+        <v>65</v>
+      </c>
+      <c r="C38" t="s">
+        <v>249</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>59</v>
+      </c>
+      <c r="B39" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" t="s">
+        <v>249</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>59</v>
+      </c>
+      <c r="B40" t="s">
+        <v>65</v>
+      </c>
+      <c r="C40" t="s">
+        <v>249</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>59</v>
+      </c>
+      <c r="B41" t="s">
+        <v>65</v>
+      </c>
+      <c r="C41" t="s">
+        <v>249</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>59</v>
+      </c>
+      <c r="B42" t="s">
+        <v>65</v>
+      </c>
+      <c r="C42" t="s">
+        <v>249</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>59</v>
+      </c>
+      <c r="B43" t="s">
+        <v>65</v>
+      </c>
+      <c r="C43" t="s">
+        <v>249</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>59</v>
+      </c>
+      <c r="B44" t="s">
+        <v>65</v>
+      </c>
+      <c r="C44" t="s">
+        <v>249</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>59</v>
+      </c>
+      <c r="B45" t="s">
+        <v>65</v>
+      </c>
+      <c r="C45" t="s">
+        <v>249</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>59</v>
+      </c>
+      <c r="B46" t="s">
+        <v>65</v>
+      </c>
+      <c r="C46" t="s">
+        <v>249</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>59</v>
+      </c>
+      <c r="B47" t="s">
+        <v>65</v>
+      </c>
+      <c r="C47" t="s">
+        <v>249</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>59</v>
+      </c>
+      <c r="B48" t="s">
+        <v>65</v>
+      </c>
+      <c r="C48" t="s">
+        <v>249</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>59</v>
+      </c>
+      <c r="B49" t="s">
+        <v>65</v>
+      </c>
+      <c r="C49" t="s">
+        <v>249</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>59</v>
+      </c>
+      <c r="B50" t="s">
+        <v>65</v>
+      </c>
+      <c r="C50" t="s">
+        <v>249</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>59</v>
+      </c>
+      <c r="B51" t="s">
+        <v>65</v>
+      </c>
+      <c r="C51" t="s">
+        <v>249</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52" t="s">
+        <v>65</v>
+      </c>
+      <c r="C52" t="s">
+        <v>249</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>59</v>
+      </c>
+      <c r="B53" t="s">
+        <v>65</v>
+      </c>
+      <c r="C53" t="s">
+        <v>249</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>59</v>
+      </c>
+      <c r="B54" t="s">
+        <v>65</v>
+      </c>
+      <c r="C54" t="s">
+        <v>249</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>59</v>
+      </c>
+      <c r="B55" t="s">
+        <v>65</v>
+      </c>
+      <c r="C55" t="s">
+        <v>249</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>59</v>
+      </c>
+      <c r="B56" t="s">
+        <v>65</v>
+      </c>
+      <c r="C56" t="s">
+        <v>249</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" t="s">
+        <v>65</v>
+      </c>
+      <c r="C57" t="s">
+        <v>249</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>59</v>
+      </c>
+      <c r="B58" t="s">
+        <v>94</v>
+      </c>
+      <c r="C58" t="s">
+        <v>250</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>59</v>
+      </c>
+      <c r="B59" t="s">
+        <v>94</v>
+      </c>
+      <c r="C59" t="s">
+        <v>250</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>94</v>
+      </c>
+      <c r="C60" t="s">
+        <v>250</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>59</v>
+      </c>
+      <c r="B61" t="s">
+        <v>94</v>
+      </c>
+      <c r="C61" t="s">
+        <v>250</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>59</v>
+      </c>
+      <c r="B62" t="s">
+        <v>94</v>
+      </c>
+      <c r="C62" t="s">
+        <v>250</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>59</v>
+      </c>
+      <c r="B63" t="s">
+        <v>94</v>
+      </c>
+      <c r="C63" t="s">
+        <v>250</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>59</v>
+      </c>
+      <c r="B64" t="s">
+        <v>94</v>
+      </c>
+      <c r="C64" t="s">
+        <v>250</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>59</v>
+      </c>
+      <c r="B65" t="s">
+        <v>94</v>
+      </c>
+      <c r="C65" t="s">
+        <v>250</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>59</v>
+      </c>
+      <c r="B66" t="s">
+        <v>94</v>
+      </c>
+      <c r="C66" t="s">
+        <v>250</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>59</v>
+      </c>
+      <c r="B67" t="s">
+        <v>94</v>
+      </c>
+      <c r="C67" t="s">
+        <v>250</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>59</v>
+      </c>
+      <c r="B68" t="s">
+        <v>94</v>
+      </c>
+      <c r="C68" t="s">
+        <v>250</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>59</v>
+      </c>
+      <c r="B69" t="s">
+        <v>106</v>
+      </c>
+      <c r="C69" t="s">
+        <v>251</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>59</v>
+      </c>
+      <c r="B70" t="s">
+        <v>106</v>
+      </c>
+      <c r="C70" t="s">
+        <v>251</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>59</v>
+      </c>
+      <c r="B71" t="s">
+        <v>106</v>
+      </c>
+      <c r="C71" t="s">
+        <v>251</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>59</v>
+      </c>
+      <c r="B72" t="s">
+        <v>106</v>
+      </c>
+      <c r="C72" t="s">
+        <v>251</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>59</v>
+      </c>
+      <c r="B73" t="s">
+        <v>106</v>
+      </c>
+      <c r="C73" t="s">
+        <v>251</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>59</v>
+      </c>
+      <c r="B74" t="s">
+        <v>106</v>
+      </c>
+      <c r="C74" t="s">
+        <v>251</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>59</v>
+      </c>
+      <c r="B75" t="s">
+        <v>106</v>
+      </c>
+      <c r="C75" t="s">
+        <v>251</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>59</v>
+      </c>
+      <c r="B76" t="s">
+        <v>106</v>
+      </c>
+      <c r="C76" t="s">
+        <v>251</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>59</v>
+      </c>
+      <c r="B77" t="s">
+        <v>115</v>
+      </c>
+      <c r="C77" t="s">
+        <v>252</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>59</v>
+      </c>
+      <c r="B78" t="s">
+        <v>115</v>
+      </c>
+      <c r="C78" t="s">
+        <v>252</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>59</v>
+      </c>
+      <c r="B79" t="s">
+        <v>115</v>
+      </c>
+      <c r="C79" t="s">
+        <v>252</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>59</v>
+      </c>
+      <c r="B80" t="s">
+        <v>115</v>
+      </c>
+      <c r="C80" t="s">
+        <v>252</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>120</v>
+      </c>
+      <c r="B81" t="s">
+        <v>121</v>
+      </c>
+      <c r="C81" t="s">
+        <v>253</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>120</v>
+      </c>
+      <c r="B82" t="s">
+        <v>121</v>
+      </c>
+      <c r="C82" t="s">
+        <v>253</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>120</v>
+      </c>
+      <c r="B83" t="s">
+        <v>121</v>
+      </c>
+      <c r="C83" t="s">
+        <v>253</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>120</v>
+      </c>
+      <c r="B84" t="s">
+        <v>121</v>
+      </c>
+      <c r="C84" t="s">
+        <v>253</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>120</v>
+      </c>
+      <c r="B85" t="s">
+        <v>121</v>
+      </c>
+      <c r="C85" t="s">
+        <v>253</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>120</v>
+      </c>
+      <c r="B86" t="s">
+        <v>121</v>
+      </c>
+      <c r="C86" t="s">
+        <v>253</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>120</v>
+      </c>
+      <c r="B87" t="s">
+        <v>121</v>
+      </c>
+      <c r="C87" t="s">
+        <v>253</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F87" s="1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>120</v>
+      </c>
+      <c r="B88" t="s">
+        <v>121</v>
+      </c>
+      <c r="C88" t="s">
+        <v>253</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>120</v>
+      </c>
+      <c r="B89" t="s">
+        <v>121</v>
+      </c>
+      <c r="C89" t="s">
+        <v>253</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>120</v>
+      </c>
+      <c r="B90" t="s">
+        <v>121</v>
+      </c>
+      <c r="C90" t="s">
+        <v>253</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>120</v>
+      </c>
+      <c r="B91" t="s">
+        <v>121</v>
+      </c>
+      <c r="C91" t="s">
+        <v>253</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92" t="s">
+        <v>133</v>
+      </c>
+      <c r="C92" t="s">
+        <v>254</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>120</v>
+      </c>
+      <c r="B93" t="s">
+        <v>133</v>
+      </c>
+      <c r="C93" t="s">
+        <v>254</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>120</v>
+      </c>
+      <c r="B94" t="s">
+        <v>133</v>
+      </c>
+      <c r="C94" t="s">
+        <v>254</v>
+      </c>
+      <c r="D94" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>120</v>
+      </c>
+      <c r="B95" t="s">
+        <v>137</v>
+      </c>
+      <c r="C95" t="s">
+        <v>255</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="F95" s="1" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>120</v>
+      </c>
+      <c r="B96" t="s">
+        <v>137</v>
+      </c>
+      <c r="C96" t="s">
+        <v>255</v>
+      </c>
+      <c r="D96" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F96" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>120</v>
+      </c>
+      <c r="B97" t="s">
+        <v>137</v>
+      </c>
+      <c r="C97" t="s">
+        <v>255</v>
+      </c>
+      <c r="D97" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F97" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>141</v>
+      </c>
+      <c r="B98" t="s">
+        <v>142</v>
+      </c>
+      <c r="C98" t="s">
+        <v>256</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F98" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>141</v>
+      </c>
+      <c r="B99" t="s">
+        <v>142</v>
+      </c>
+      <c r="C99" t="s">
+        <v>256</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="F99" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>141</v>
+      </c>
+      <c r="B100" t="s">
+        <v>142</v>
+      </c>
+      <c r="C100" t="s">
+        <v>256</v>
+      </c>
+      <c r="D100" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F100" s="1" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>141</v>
+      </c>
+      <c r="B101" t="s">
+        <v>142</v>
+      </c>
+      <c r="C101" t="s">
+        <v>256</v>
+      </c>
+      <c r="D101" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F101" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>141</v>
+      </c>
+      <c r="B102" t="s">
+        <v>147</v>
+      </c>
+      <c r="C102" t="s">
+        <v>257</v>
+      </c>
+      <c r="D102" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="F102" s="1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>141</v>
+      </c>
+      <c r="B103" t="s">
+        <v>147</v>
+      </c>
+      <c r="C103" t="s">
+        <v>257</v>
+      </c>
+      <c r="D103" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -2260,15 +4438,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101007DF10FFD192FFC4D8577319E294160E1" ma:contentTypeVersion="4" ma:contentTypeDescription="Vytvoří nový dokument" ma:contentTypeScope="" ma:versionID="173bbea147869ab09aeda7c02d1f1dc8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2f9db504-8788-409d-aff0-8874d63f73c0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b81c9415cca2b8e1e97e24443b05ecbe" ns2:_="">
     <xsd:import namespace="2f9db504-8788-409d-aff0-8874d63f73c0"/>
@@ -2412,6 +4581,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -2419,15 +4597,38 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1522E275-4BA9-45DA-B292-83106A295751}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75DC23A1-8D5B-43ED-9FEB-E940D051E2D2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2f9db504-8788-409d-aff0-8874d63f73c0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75DC23A1-8D5B-43ED-9FEB-E940D051E2D2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1522E275-4BA9-45DA-B292-83106A295751}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0CACC73-48CD-4204-9397-82C618DB3D42}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0CACC73-48CD-4204-9397-82C618DB3D42}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>